<commit_message>
Посты Instagram и Telegram: 2026-10-05
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -25,8 +25,8 @@
     <numFmt numFmtId="165" formatCode="0.0%;\-0.0%;0.0%"/>
     <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="169" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="168" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -215,7 +215,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -334,7 +334,7 @@
     <xf numFmtId="3" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
@@ -351,7 +351,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="169" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -363,10 +363,15 @@
     <xf numFmtId="167" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="169" fontId="18" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="18" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -493,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$3</f>
+              <f>'Динамика'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$3</f>
+              <f>'Динамика'!$B$2:$B$4</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1577,14 +1582,21 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="40" t="n">
+      <c r="A3" s="55" t="n">
         <v>46299</v>
       </c>
       <c r="B3" s="41" t="n">
         <v>3226</v>
       </c>
     </row>
-    <row r="4"/>
+    <row r="4">
+      <c r="A4" s="55" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B4" s="41" t="n">
+        <v>3226</v>
+      </c>
+    </row>
     <row r="5"/>
     <row r="6"/>
     <row r="7"/>
@@ -3131,7 +3143,7 @@
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="25">
-      <c r="A2" s="47" t="n">
+      <c r="A2" s="56" t="n">
         <v>46297</v>
       </c>
       <c r="B2" s="48" t="inlineStr">
@@ -3177,12 +3189,12 @@
         <f>IF(N(G2)&gt;0,(I2+J2+K2+L2)/G2,"")</f>
         <v/>
       </c>
-      <c r="N2" s="47" t="n">
-        <v>46299</v>
+      <c r="N2" s="56" t="n">
+        <v>46301</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="51" t="n">
+      <c r="A3" s="57" t="n">
         <v>46299</v>
       </c>
       <c r="B3" s="52" t="inlineStr">
@@ -3207,13 +3219,13 @@
         </is>
       </c>
       <c r="G3" s="52" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="H3" s="52" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="I3" s="52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" s="52" t="n">
         <v>0</v>
@@ -3228,8 +3240,8 @@
         <f>IF(N(G3)&gt;0,(I3+J3+K3+L3)/G3,"")</f>
         <v/>
       </c>
-      <c r="N3" s="51" t="n">
-        <v>46299</v>
+      <c r="N3" s="57" t="n">
+        <v>46301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-07
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$4</f>
+              <f>'Динамика'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$4</f>
+              <f>'Динамика'!$B$2:$B$5</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -676,12 +676,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Наши посты'!$B$2:$B$3</f>
+              <f>'Наши посты'!$B$2:$B$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Наши посты'!$G$2:$G$3</f>
+              <f>'Наши посты'!$G$2:$G$4</f>
             </numRef>
           </val>
         </ser>
@@ -1597,7 +1597,14 @@
         <v>3226</v>
       </c>
     </row>
-    <row r="5"/>
+    <row r="5">
+      <c r="A5" s="55" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B5" s="41" t="n">
+        <v>3225</v>
+      </c>
+    </row>
     <row r="6"/>
     <row r="7"/>
     <row r="8"/>
@@ -3053,7 +3060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3168,10 +3175,10 @@
         </is>
       </c>
       <c r="G2" s="48" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H2" s="48" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="I2" s="48" t="n">
         <v>3</v>
@@ -3190,7 +3197,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="3">
@@ -3219,10 +3226,10 @@
         </is>
       </c>
       <c r="G3" s="52" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H3" s="52" t="n">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="I3" s="52" t="n">
         <v>1</v>
@@ -3241,13 +3248,65 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46301</v>
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="57" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>p04</t>
+        </is>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t>Утеплённые школьные брюки палаццо</t>
+        </is>
+      </c>
+      <c r="D4" s="52" t="n">
+        <v>481319471</v>
+      </c>
+      <c r="E4" s="52" t="n">
+        <v>2581693697</v>
+      </c>
+      <c r="F4" s="53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/DeNP7SDDVXc/</t>
+        </is>
+      </c>
+      <c r="G4" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="54">
+        <f>IF(N(G4)&gt;0,(I4+J4+K4+L4)/G4,"")</f>
+        <v/>
+      </c>
+      <c r="N4" s="57" t="n">
+        <v>46302</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-09
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$5</f>
+              <f>'Динамика'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$5</f>
+              <f>'Динамика'!$B$2:$B$6</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -676,12 +676,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Наши посты'!$B$2:$B$4</f>
+              <f>'Наши посты'!$B$2:$B$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Наши посты'!$G$2:$G$4</f>
+              <f>'Наши посты'!$G$2:$G$5</f>
             </numRef>
           </val>
         </ser>
@@ -1605,7 +1605,14 @@
         <v>3225</v>
       </c>
     </row>
-    <row r="6"/>
+    <row r="6">
+      <c r="A6" s="55" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B6" s="41" t="n">
+        <v>3227</v>
+      </c>
+    </row>
     <row r="7"/>
     <row r="8"/>
     <row r="9"/>
@@ -3060,7 +3067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3175,10 +3182,10 @@
         </is>
       </c>
       <c r="G2" s="48" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H2" s="48" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I2" s="48" t="n">
         <v>3</v>
@@ -3197,7 +3204,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46302</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="3">
@@ -3226,13 +3233,13 @@
         </is>
       </c>
       <c r="G3" s="52" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H3" s="52" t="n">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="I3" s="52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3" s="52" t="n">
         <v>0</v>
@@ -3248,7 +3255,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46302</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="4">
@@ -3277,13 +3284,13 @@
         </is>
       </c>
       <c r="G4" s="52" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="H4" s="52" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="I4" s="52" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J4" s="52" t="n">
         <v>0</v>
@@ -3299,7 +3306,58 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46302</v>
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="57" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B5" s="52" t="inlineStr">
+        <is>
+          <t>p05</t>
+        </is>
+      </c>
+      <c r="C5" s="52" t="inlineStr">
+        <is>
+          <t>Костюм для девочки с принтом</t>
+        </is>
+      </c>
+      <c r="D5" s="52" t="n">
+        <v>479961106</v>
+      </c>
+      <c r="E5" s="52" t="n">
+        <v>2581089081</v>
+      </c>
+      <c r="F5" s="53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DeSWbZgmSyf/</t>
+        </is>
+      </c>
+      <c r="G5" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="54">
+        <f>IF(N(G5)&gt;0,(I5+J5+K5+L5)/G5,"")</f>
+        <v/>
+      </c>
+      <c r="N5" s="57" t="n">
+        <v>46304</v>
       </c>
     </row>
   </sheetData>
@@ -3307,6 +3365,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-11
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$6</f>
+              <f>'Динамика'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$6</f>
+              <f>'Динамика'!$B$2:$B$7</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -676,12 +676,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Наши посты'!$B$2:$B$5</f>
+              <f>'Наши посты'!$B$2:$B$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Наши посты'!$G$2:$G$5</f>
+              <f>'Наши посты'!$G$2:$G$6</f>
             </numRef>
           </val>
         </ser>
@@ -1613,7 +1613,14 @@
         <v>3227</v>
       </c>
     </row>
-    <row r="7"/>
+    <row r="7">
+      <c r="A7" s="55" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B7" s="41" t="n">
+        <v>3228</v>
+      </c>
+    </row>
     <row r="8"/>
     <row r="9"/>
     <row r="10"/>
@@ -3067,7 +3074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3182,10 +3189,10 @@
         </is>
       </c>
       <c r="G2" s="48" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H2" s="48" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I2" s="48" t="n">
         <v>3</v>
@@ -3204,7 +3211,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46304</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="3">
@@ -3233,13 +3240,13 @@
         </is>
       </c>
       <c r="G3" s="52" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="H3" s="52" t="n">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="I3" s="52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J3" s="52" t="n">
         <v>0</v>
@@ -3255,7 +3262,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46304</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="4">
@@ -3284,10 +3291,10 @@
         </is>
       </c>
       <c r="G4" s="52" t="n">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="H4" s="52" t="n">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="I4" s="52" t="n">
         <v>3</v>
@@ -3306,7 +3313,7 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46304</v>
+        <v>46306</v>
       </c>
     </row>
     <row r="5">
@@ -3335,13 +3342,13 @@
         </is>
       </c>
       <c r="G5" s="52" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="H5" s="52" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="I5" s="52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" s="52" t="n">
         <v>0</v>
@@ -3357,7 +3364,58 @@
         <v/>
       </c>
       <c r="N5" s="57" t="n">
-        <v>46304</v>
+        <v>46306</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="57" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B6" s="52" t="inlineStr">
+        <is>
+          <t>p06</t>
+        </is>
+      </c>
+      <c r="C6" s="52" t="inlineStr">
+        <is>
+          <t>Тёплый костюм для девочки — 4 оттенка</t>
+        </is>
+      </c>
+      <c r="D6" s="52" t="n">
+        <v>22061090</v>
+      </c>
+      <c r="E6" s="52" t="n">
+        <v>856765298</v>
+      </c>
+      <c r="F6" s="53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DeXbwysGDVs/</t>
+        </is>
+      </c>
+      <c r="G6" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="54">
+        <f>IF(N(G6)&gt;0,(I6+J6+K6+L6)/G6,"")</f>
+        <v/>
+      </c>
+      <c r="N6" s="57" t="n">
+        <v>46306</v>
       </c>
     </row>
   </sheetData>
@@ -3366,6 +3424,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-12
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$7</f>
+              <f>'Динамика'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$7</f>
+              <f>'Динамика'!$B$2:$B$8</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1621,7 +1621,14 @@
         <v>3228</v>
       </c>
     </row>
-    <row r="8"/>
+    <row r="8">
+      <c r="A8" s="55" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B8" s="41" t="n">
+        <v>3228</v>
+      </c>
+    </row>
     <row r="9"/>
     <row r="10"/>
     <row r="11"/>
@@ -3211,7 +3218,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="3">
@@ -3240,10 +3247,10 @@
         </is>
       </c>
       <c r="G3" s="52" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H3" s="52" t="n">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="I3" s="52" t="n">
         <v>3</v>
@@ -3262,7 +3269,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="4">
@@ -3291,10 +3298,10 @@
         </is>
       </c>
       <c r="G4" s="52" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H4" s="52" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="I4" s="52" t="n">
         <v>3</v>
@@ -3313,7 +3320,7 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="5">
@@ -3342,10 +3349,10 @@
         </is>
       </c>
       <c r="G5" s="52" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H5" s="52" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="I5" s="52" t="n">
         <v>1</v>
@@ -3364,7 +3371,7 @@
         <v/>
       </c>
       <c r="N5" s="57" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="6">
@@ -3393,10 +3400,10 @@
         </is>
       </c>
       <c r="G6" s="52" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="H6" s="52" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="I6" s="52" t="n">
         <v>0</v>
@@ -3415,7 +3422,7 @@
         <v/>
       </c>
       <c r="N6" s="57" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-14
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$8</f>
+              <f>'Динамика'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$8</f>
+              <f>'Динамика'!$B$2:$B$9</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1629,7 +1629,14 @@
         <v>3228</v>
       </c>
     </row>
-    <row r="9"/>
+    <row r="9">
+      <c r="A9" s="55" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B9" s="41" t="n">
+        <v>3227</v>
+      </c>
+    </row>
     <row r="10"/>
     <row r="11"/>
     <row r="12"/>
@@ -3218,7 +3225,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="3">
@@ -3247,10 +3254,10 @@
         </is>
       </c>
       <c r="G3" s="52" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H3" s="52" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="I3" s="52" t="n">
         <v>3</v>
@@ -3269,7 +3276,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="4">
@@ -3298,10 +3305,10 @@
         </is>
       </c>
       <c r="G4" s="52" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H4" s="52" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="I4" s="52" t="n">
         <v>3</v>
@@ -3320,7 +3327,7 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="5">
@@ -3349,10 +3356,10 @@
         </is>
       </c>
       <c r="G5" s="52" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H5" s="52" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="I5" s="52" t="n">
         <v>1</v>
@@ -3371,7 +3378,7 @@
         <v/>
       </c>
       <c r="N5" s="57" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="6">
@@ -3400,10 +3407,10 @@
         </is>
       </c>
       <c r="G6" s="52" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="H6" s="52" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="I6" s="52" t="n">
         <v>0</v>
@@ -3422,7 +3429,7 @@
         <v/>
       </c>
       <c r="N6" s="57" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-16
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$9</f>
+              <f>'Динамика'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$9</f>
+              <f>'Динамика'!$B$2:$B$10</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -676,12 +676,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Наши посты'!$B$2:$B$7</f>
+              <f>'Наши посты'!$B$2:$B$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Наши посты'!$G$2:$G$7</f>
+              <f>'Наши посты'!$G$2:$G$8</f>
             </numRef>
           </val>
         </ser>
@@ -1637,7 +1637,14 @@
         <v>3227</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10">
+      <c r="A10" s="55" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B10" s="41" t="n">
+        <v>3227</v>
+      </c>
+    </row>
     <row r="11"/>
     <row r="12"/>
     <row r="13"/>
@@ -3088,7 +3095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3203,10 +3210,10 @@
         </is>
       </c>
       <c r="G2" s="48" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H2" s="48" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I2" s="48" t="n">
         <v>3</v>
@@ -3225,7 +3232,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="3">
@@ -3254,10 +3261,10 @@
         </is>
       </c>
       <c r="G3" s="52" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H3" s="52" t="n">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="I3" s="52" t="n">
         <v>3</v>
@@ -3276,7 +3283,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="4">
@@ -3305,13 +3312,13 @@
         </is>
       </c>
       <c r="G4" s="52" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H4" s="52" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I4" s="52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J4" s="52" t="n">
         <v>0</v>
@@ -3327,7 +3334,7 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="5">
@@ -3356,13 +3363,13 @@
         </is>
       </c>
       <c r="G5" s="52" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="H5" s="52" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="I5" s="52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" s="52" t="n">
         <v>0</v>
@@ -3378,7 +3385,7 @@
         <v/>
       </c>
       <c r="N5" s="57" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="6">
@@ -3407,10 +3414,10 @@
         </is>
       </c>
       <c r="G6" s="52" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="H6" s="52" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="I6" s="52" t="n">
         <v>0</v>
@@ -3429,7 +3436,7 @@
         <v/>
       </c>
       <c r="N6" s="57" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="7">
@@ -3458,10 +3465,10 @@
         </is>
       </c>
       <c r="G7" s="52" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="H7" s="52" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="I7" s="52" t="n">
         <v>0</v>
@@ -3480,7 +3487,58 @@
         <v/>
       </c>
       <c r="N7" s="57" t="n">
-        <v>46309</v>
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="57" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B8" s="52" t="inlineStr">
+        <is>
+          <t>p09</t>
+        </is>
+      </c>
+      <c r="C8" s="52" t="inlineStr">
+        <is>
+          <t>Спортивный костюм со шнуровкой</t>
+        </is>
+      </c>
+      <c r="D8" s="52" t="n">
+        <v>124002921</v>
+      </c>
+      <c r="E8" s="52" t="n">
+        <v>855854788</v>
+      </c>
+      <c r="F8" s="53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DekO47WlkVn/</t>
+        </is>
+      </c>
+      <c r="G8" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="54">
+        <f>IF(N(G8)&gt;0,(I8+J8+K8+L8)/G8,"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="57" t="n">
+        <v>46311</v>
       </c>
     </row>
   </sheetData>
@@ -3491,6 +3549,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-18
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$10</f>
+              <f>'Динамика'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$10</f>
+              <f>'Динамика'!$B$2:$B$11</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -676,12 +676,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Наши посты'!$B$2:$B$8</f>
+              <f>'Наши посты'!$B$2:$B$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Наши посты'!$G$2:$G$8</f>
+              <f>'Наши посты'!$G$2:$G$9</f>
             </numRef>
           </val>
         </ser>
@@ -1645,7 +1645,14 @@
         <v>3227</v>
       </c>
     </row>
-    <row r="11"/>
+    <row r="11">
+      <c r="A11" s="55" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B11" s="41" t="n">
+        <v>3226</v>
+      </c>
+    </row>
     <row r="12"/>
     <row r="13"/>
     <row r="14"/>
@@ -3095,7 +3102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3232,7 +3239,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="3">
@@ -3283,7 +3290,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="4">
@@ -3312,10 +3319,10 @@
         </is>
       </c>
       <c r="G4" s="52" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="H4" s="52" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="I4" s="52" t="n">
         <v>4</v>
@@ -3334,7 +3341,7 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="5">
@@ -3363,10 +3370,10 @@
         </is>
       </c>
       <c r="G5" s="52" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H5" s="52" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="I5" s="52" t="n">
         <v>2</v>
@@ -3385,7 +3392,7 @@
         <v/>
       </c>
       <c r="N5" s="57" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="6">
@@ -3414,10 +3421,10 @@
         </is>
       </c>
       <c r="G6" s="52" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H6" s="52" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I6" s="52" t="n">
         <v>0</v>
@@ -3436,7 +3443,7 @@
         <v/>
       </c>
       <c r="N6" s="57" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="7">
@@ -3465,10 +3472,10 @@
         </is>
       </c>
       <c r="G7" s="52" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="H7" s="52" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="I7" s="52" t="n">
         <v>0</v>
@@ -3487,7 +3494,7 @@
         <v/>
       </c>
       <c r="N7" s="57" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="8">
@@ -3516,13 +3523,13 @@
         </is>
       </c>
       <c r="G8" s="52" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H8" s="52" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I8" s="52" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J8" s="52" t="n">
         <v>0</v>
@@ -3538,7 +3545,58 @@
         <v/>
       </c>
       <c r="N8" s="57" t="n">
-        <v>46311</v>
+        <v>46313</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="57" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B9" s="52" t="inlineStr">
+        <is>
+          <t>p10</t>
+        </is>
+      </c>
+      <c r="C9" s="52" t="inlineStr">
+        <is>
+          <t>Костюм с начёсом и принтом на спине</t>
+        </is>
+      </c>
+      <c r="D9" s="52" t="n">
+        <v>502796956</v>
+      </c>
+      <c r="E9" s="52" t="n">
+        <v>2775992327</v>
+      </c>
+      <c r="F9" s="53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DepTivqnCbC/</t>
+        </is>
+      </c>
+      <c r="G9" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="54">
+        <f>IF(N(G9)&gt;0,(I9+J9+K9+L9)/G9,"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="57" t="n">
+        <v>46313</v>
       </c>
     </row>
   </sheetData>
@@ -3550,6 +3608,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-19
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$11</f>
+              <f>'Динамика'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$11</f>
+              <f>'Динамика'!$B$2:$B$12</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -676,12 +676,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Наши посты'!$B$2:$B$9</f>
+              <f>'Наши посты'!$B$2:$B$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Наши посты'!$G$2:$G$9</f>
+              <f>'Наши посты'!$G$2:$G$10</f>
             </numRef>
           </val>
         </ser>
@@ -1653,7 +1653,14 @@
         <v>3226</v>
       </c>
     </row>
-    <row r="12"/>
+    <row r="12">
+      <c r="A12" s="55" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B12" s="41" t="n">
+        <v>3226</v>
+      </c>
+    </row>
     <row r="13"/>
     <row r="14"/>
     <row r="15"/>
@@ -3102,7 +3109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3239,7 +3246,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="3">
@@ -3290,7 +3297,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="4">
@@ -3341,7 +3348,7 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="5">
@@ -3392,7 +3399,7 @@
         <v/>
       </c>
       <c r="N5" s="57" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="6">
@@ -3421,10 +3428,10 @@
         </is>
       </c>
       <c r="G6" s="52" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H6" s="52" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="I6" s="52" t="n">
         <v>0</v>
@@ -3443,7 +3450,7 @@
         <v/>
       </c>
       <c r="N6" s="57" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="7">
@@ -3472,10 +3479,10 @@
         </is>
       </c>
       <c r="G7" s="52" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="H7" s="52" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I7" s="52" t="n">
         <v>0</v>
@@ -3494,7 +3501,7 @@
         <v/>
       </c>
       <c r="N7" s="57" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="8">
@@ -3523,10 +3530,10 @@
         </is>
       </c>
       <c r="G8" s="52" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="H8" s="52" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="I8" s="52" t="n">
         <v>2</v>
@@ -3545,7 +3552,7 @@
         <v/>
       </c>
       <c r="N8" s="57" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="9">
@@ -3574,13 +3581,13 @@
         </is>
       </c>
       <c r="G9" s="52" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H9" s="52" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I9" s="52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" s="52" t="n">
         <v>0</v>
@@ -3596,7 +3603,58 @@
         <v/>
       </c>
       <c r="N9" s="57" t="n">
-        <v>46313</v>
+        <v>46314</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="57" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B10" s="52" t="inlineStr">
+        <is>
+          <t>p11</t>
+        </is>
+      </c>
+      <c r="C10" s="52" t="inlineStr">
+        <is>
+          <t>Тёплый костюм для мальчика с принтом</t>
+        </is>
+      </c>
+      <c r="D10" s="52" t="n">
+        <v>493757862</v>
+      </c>
+      <c r="E10" s="52" t="n">
+        <v>2717792134</v>
+      </c>
+      <c r="F10" s="53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DesJDEuiRm8/</t>
+        </is>
+      </c>
+      <c r="G10" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="54">
+        <f>IF(N(G10)&gt;0,(I10+J10+K10+L10)/G10,"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="57" t="n">
+        <v>46314</v>
       </c>
     </row>
   </sheetData>
@@ -3609,6 +3667,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-21
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$12</f>
+              <f>'Динамика'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$12</f>
+              <f>'Динамика'!$B$2:$B$13</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -676,12 +676,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Наши посты'!$B$2:$B$10</f>
+              <f>'Наши посты'!$B$2:$B$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Наши посты'!$G$2:$G$10</f>
+              <f>'Наши посты'!$G$2:$G$11</f>
             </numRef>
           </val>
         </ser>
@@ -1661,7 +1661,14 @@
         <v>3226</v>
       </c>
     </row>
-    <row r="13"/>
+    <row r="13">
+      <c r="A13" s="55" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B13" s="41" t="n">
+        <v>3225</v>
+      </c>
+    </row>
     <row r="14"/>
     <row r="15"/>
     <row r="16"/>
@@ -3109,7 +3116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3246,7 +3253,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="3">
@@ -3297,7 +3304,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="4">
@@ -3348,7 +3355,7 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="5">
@@ -3377,10 +3384,10 @@
         </is>
       </c>
       <c r="G5" s="52" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H5" s="52" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I5" s="52" t="n">
         <v>2</v>
@@ -3399,7 +3406,7 @@
         <v/>
       </c>
       <c r="N5" s="57" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="6">
@@ -3450,7 +3457,7 @@
         <v/>
       </c>
       <c r="N6" s="57" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="7">
@@ -3479,10 +3486,10 @@
         </is>
       </c>
       <c r="G7" s="52" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H7" s="52" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I7" s="52" t="n">
         <v>0</v>
@@ -3501,7 +3508,7 @@
         <v/>
       </c>
       <c r="N7" s="57" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="8">
@@ -3530,10 +3537,10 @@
         </is>
       </c>
       <c r="G8" s="52" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="H8" s="52" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="I8" s="52" t="n">
         <v>2</v>
@@ -3552,7 +3559,7 @@
         <v/>
       </c>
       <c r="N8" s="57" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="9">
@@ -3581,10 +3588,10 @@
         </is>
       </c>
       <c r="G9" s="52" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="H9" s="52" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I9" s="52" t="n">
         <v>1</v>
@@ -3603,7 +3610,7 @@
         <v/>
       </c>
       <c r="N9" s="57" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="10">
@@ -3632,13 +3639,13 @@
         </is>
       </c>
       <c r="G10" s="52" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H10" s="52" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I10" s="52" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J10" s="52" t="n">
         <v>0</v>
@@ -3647,14 +3654,65 @@
         <v>0</v>
       </c>
       <c r="L10" s="52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10" s="54">
         <f>IF(N(G10)&gt;0,(I10+J10+K10+L10)/G10,"")</f>
         <v/>
       </c>
       <c r="N10" s="57" t="n">
-        <v>46314</v>
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="57" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B11" s="52" t="inlineStr">
+        <is>
+          <t>p12</t>
+        </is>
+      </c>
+      <c r="C11" s="52" t="inlineStr">
+        <is>
+          <t>Тёплый костюм с капюшоном: 7 цветов</t>
+        </is>
+      </c>
+      <c r="D11" s="52" t="n">
+        <v>88668054</v>
+      </c>
+      <c r="E11" s="52" t="n">
+        <v>857790934</v>
+      </c>
+      <c r="F11" s="53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/DexK31oAuYN/</t>
+        </is>
+      </c>
+      <c r="G11" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="54">
+        <f>IF(N(G11)&gt;0,(I11+J11+K11+L11)/G11,"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="57" t="n">
+        <v>46316</v>
       </c>
     </row>
   </sheetData>
@@ -3668,6 +3726,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-23
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$13</f>
+              <f>'Динамика'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$13</f>
+              <f>'Динамика'!$B$2:$B$14</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -676,12 +676,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Наши посты'!$B$2:$B$11</f>
+              <f>'Наши посты'!$B$2:$B$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Наши посты'!$G$2:$G$11</f>
+              <f>'Наши посты'!$G$2:$G$12</f>
             </numRef>
           </val>
         </ser>
@@ -1669,7 +1669,14 @@
         <v>3225</v>
       </c>
     </row>
-    <row r="14"/>
+    <row r="14">
+      <c r="A14" s="55" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B14" s="41" t="n">
+        <v>3227</v>
+      </c>
+    </row>
     <row r="15"/>
     <row r="16"/>
     <row r="17"/>
@@ -3116,7 +3123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3253,7 +3260,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="3">
@@ -3304,7 +3311,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="4">
@@ -3355,7 +3362,7 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="5">
@@ -3384,10 +3391,10 @@
         </is>
       </c>
       <c r="G5" s="52" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H5" s="52" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="I5" s="52" t="n">
         <v>2</v>
@@ -3406,7 +3413,7 @@
         <v/>
       </c>
       <c r="N5" s="57" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="6">
@@ -3435,10 +3442,10 @@
         </is>
       </c>
       <c r="G6" s="52" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H6" s="52" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I6" s="52" t="n">
         <v>0</v>
@@ -3457,7 +3464,7 @@
         <v/>
       </c>
       <c r="N6" s="57" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="7">
@@ -3486,10 +3493,10 @@
         </is>
       </c>
       <c r="G7" s="52" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H7" s="52" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I7" s="52" t="n">
         <v>0</v>
@@ -3508,7 +3515,7 @@
         <v/>
       </c>
       <c r="N7" s="57" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="8">
@@ -3537,10 +3544,10 @@
         </is>
       </c>
       <c r="G8" s="52" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H8" s="52" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="I8" s="52" t="n">
         <v>2</v>
@@ -3559,7 +3566,7 @@
         <v/>
       </c>
       <c r="N8" s="57" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="9">
@@ -3588,10 +3595,10 @@
         </is>
       </c>
       <c r="G9" s="52" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H9" s="52" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I9" s="52" t="n">
         <v>1</v>
@@ -3610,7 +3617,7 @@
         <v/>
       </c>
       <c r="N9" s="57" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="10">
@@ -3639,10 +3646,10 @@
         </is>
       </c>
       <c r="G10" s="52" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H10" s="52" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="I10" s="52" t="n">
         <v>3</v>
@@ -3661,7 +3668,7 @@
         <v/>
       </c>
       <c r="N10" s="57" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="11">
@@ -3690,13 +3697,13 @@
         </is>
       </c>
       <c r="G11" s="52" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="H11" s="52" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="I11" s="52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" s="52" t="n">
         <v>0</v>
@@ -3712,7 +3719,58 @@
         <v/>
       </c>
       <c r="N11" s="57" t="n">
-        <v>46316</v>
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="57" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B12" s="52" t="inlineStr">
+        <is>
+          <t>p13</t>
+        </is>
+      </c>
+      <c r="C12" s="52" t="inlineStr">
+        <is>
+          <t>Шпаргалка: как выбрать размер</t>
+        </is>
+      </c>
+      <c r="D12" s="52" t="n">
+        <v>52456955</v>
+      </c>
+      <c r="E12" s="52" t="n">
+        <v>855854486</v>
+      </c>
+      <c r="F12" s="53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/De2UHsaoH-M/</t>
+        </is>
+      </c>
+      <c r="G12" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="54">
+        <f>IF(N(G12)&gt;0,(I12+J12+K12+L12)/G12,"")</f>
+        <v/>
+      </c>
+      <c r="N12" s="57" t="n">
+        <v>46318</v>
       </c>
     </row>
   </sheetData>
@@ -3727,6 +3785,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId11"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-25
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$14</f>
+              <f>'Динамика'!$A$2:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$14</f>
+              <f>'Динамика'!$B$2:$B$15</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -676,12 +676,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Наши посты'!$B$2:$B$12</f>
+              <f>'Наши посты'!$B$2:$B$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Наши посты'!$G$2:$G$12</f>
+              <f>'Наши посты'!$G$2:$G$13</f>
             </numRef>
           </val>
         </ser>
@@ -1677,7 +1677,14 @@
         <v>3227</v>
       </c>
     </row>
-    <row r="15"/>
+    <row r="15">
+      <c r="A15" s="55" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B15" s="41" t="n">
+        <v>3226</v>
+      </c>
+    </row>
     <row r="16"/>
     <row r="17"/>
     <row r="18"/>
@@ -3123,7 +3130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3260,7 +3267,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46318</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="3">
@@ -3311,7 +3318,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46318</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="4">
@@ -3362,7 +3369,7 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46318</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="5">
@@ -3413,7 +3420,7 @@
         <v/>
       </c>
       <c r="N5" s="57" t="n">
-        <v>46318</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="6">
@@ -3442,10 +3449,10 @@
         </is>
       </c>
       <c r="G6" s="52" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H6" s="52" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="I6" s="52" t="n">
         <v>0</v>
@@ -3464,7 +3471,7 @@
         <v/>
       </c>
       <c r="N6" s="57" t="n">
-        <v>46318</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="7">
@@ -3515,7 +3522,7 @@
         <v/>
       </c>
       <c r="N7" s="57" t="n">
-        <v>46318</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="8">
@@ -3544,10 +3551,10 @@
         </is>
       </c>
       <c r="G8" s="52" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H8" s="52" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="I8" s="52" t="n">
         <v>2</v>
@@ -3566,7 +3573,7 @@
         <v/>
       </c>
       <c r="N8" s="57" t="n">
-        <v>46318</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="9">
@@ -3595,10 +3602,10 @@
         </is>
       </c>
       <c r="G9" s="52" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H9" s="52" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="I9" s="52" t="n">
         <v>1</v>
@@ -3617,7 +3624,7 @@
         <v/>
       </c>
       <c r="N9" s="57" t="n">
-        <v>46318</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="10">
@@ -3646,10 +3653,10 @@
         </is>
       </c>
       <c r="G10" s="52" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="H10" s="52" t="n">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="I10" s="52" t="n">
         <v>3</v>
@@ -3668,7 +3675,7 @@
         <v/>
       </c>
       <c r="N10" s="57" t="n">
-        <v>46318</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="11">
@@ -3697,10 +3704,10 @@
         </is>
       </c>
       <c r="G11" s="52" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H11" s="52" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="I11" s="52" t="n">
         <v>1</v>
@@ -3719,7 +3726,7 @@
         <v/>
       </c>
       <c r="N11" s="57" t="n">
-        <v>46318</v>
+        <v>46320</v>
       </c>
     </row>
     <row r="12">
@@ -3748,10 +3755,10 @@
         </is>
       </c>
       <c r="G12" s="52" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="H12" s="52" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="I12" s="52" t="n">
         <v>0</v>
@@ -3770,7 +3777,58 @@
         <v/>
       </c>
       <c r="N12" s="57" t="n">
-        <v>46318</v>
+        <v>46320</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="57" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B13" s="52" t="inlineStr">
+        <is>
+          <t>p14</t>
+        </is>
+      </c>
+      <c r="C13" s="52" t="inlineStr">
+        <is>
+          <t>Толстовка с начёсом для девочки</t>
+        </is>
+      </c>
+      <c r="D13" s="52" t="n">
+        <v>34564033</v>
+      </c>
+      <c r="E13" s="52" t="n">
+        <v>955444538</v>
+      </c>
+      <c r="F13" s="53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/De7W_jNGNKQ/</t>
+        </is>
+      </c>
+      <c r="G13" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="54">
+        <f>IF(N(G13)&gt;0,(I13+J13+K13+L13)/G13,"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="57" t="n">
+        <v>46320</v>
       </c>
     </row>
   </sheetData>
@@ -3786,6 +3844,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId12"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-26
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$15</f>
+              <f>'Динамика'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$15</f>
+              <f>'Динамика'!$B$2:$B$16</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -676,12 +676,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Наши посты'!$B$2:$B$13</f>
+              <f>'Наши посты'!$B$2:$B$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Наши посты'!$G$2:$G$13</f>
+              <f>'Наши посты'!$G$2:$G$14</f>
             </numRef>
           </val>
         </ser>
@@ -1685,7 +1685,14 @@
         <v>3226</v>
       </c>
     </row>
-    <row r="16"/>
+    <row r="16">
+      <c r="A16" s="55" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B16" s="41" t="n">
+        <v>3224</v>
+      </c>
+    </row>
     <row r="17"/>
     <row r="18"/>
     <row r="19"/>
@@ -3130,7 +3137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3267,7 +3274,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="3">
@@ -3318,7 +3325,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="4">
@@ -3369,7 +3376,7 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="5">
@@ -3420,7 +3427,7 @@
         <v/>
       </c>
       <c r="N5" s="57" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="6">
@@ -3471,7 +3478,7 @@
         <v/>
       </c>
       <c r="N6" s="57" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="7">
@@ -3522,7 +3529,7 @@
         <v/>
       </c>
       <c r="N7" s="57" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="8">
@@ -3573,7 +3580,7 @@
         <v/>
       </c>
       <c r="N8" s="57" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="9">
@@ -3602,10 +3609,10 @@
         </is>
       </c>
       <c r="G9" s="52" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H9" s="52" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I9" s="52" t="n">
         <v>1</v>
@@ -3624,7 +3631,7 @@
         <v/>
       </c>
       <c r="N9" s="57" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="10">
@@ -3653,10 +3660,10 @@
         </is>
       </c>
       <c r="G10" s="52" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H10" s="52" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="I10" s="52" t="n">
         <v>3</v>
@@ -3675,7 +3682,7 @@
         <v/>
       </c>
       <c r="N10" s="57" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="11">
@@ -3704,10 +3711,10 @@
         </is>
       </c>
       <c r="G11" s="52" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H11" s="52" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I11" s="52" t="n">
         <v>1</v>
@@ -3726,7 +3733,7 @@
         <v/>
       </c>
       <c r="N11" s="57" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="12">
@@ -3755,10 +3762,10 @@
         </is>
       </c>
       <c r="G12" s="52" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H12" s="52" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I12" s="52" t="n">
         <v>0</v>
@@ -3777,7 +3784,7 @@
         <v/>
       </c>
       <c r="N12" s="57" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="13">
@@ -3806,10 +3813,10 @@
         </is>
       </c>
       <c r="G13" s="52" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="H13" s="52" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="I13" s="52" t="n">
         <v>0</v>
@@ -3828,7 +3835,58 @@
         <v/>
       </c>
       <c r="N13" s="57" t="n">
-        <v>46320</v>
+        <v>46321</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="57" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B14" s="52" t="inlineStr">
+        <is>
+          <t>p15</t>
+        </is>
+      </c>
+      <c r="C14" s="52" t="inlineStr">
+        <is>
+          <t>Тёплые брюки с начёсом для школы</t>
+        </is>
+      </c>
+      <c r="D14" s="52" t="n">
+        <v>116569962</v>
+      </c>
+      <c r="E14" s="52" t="n">
+        <v>851169336</v>
+      </c>
+      <c r="F14" s="53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/De-K0_YGngQ/</t>
+        </is>
+      </c>
+      <c r="G14" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="54">
+        <f>IF(N(G14)&gt;0,(I14+J14+K14+L14)/G14,"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="57" t="n">
+        <v>46321</v>
       </c>
     </row>
   </sheetData>
@@ -3845,6 +3903,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId13"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-28
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$16</f>
+              <f>'Динамика'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$16</f>
+              <f>'Динамика'!$B$2:$B$17</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -676,12 +676,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Наши посты'!$B$2:$B$14</f>
+              <f>'Наши посты'!$B$2:$B$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Наши посты'!$G$2:$G$14</f>
+              <f>'Наши посты'!$G$2:$G$15</f>
             </numRef>
           </val>
         </ser>
@@ -1693,7 +1693,14 @@
         <v>3224</v>
       </c>
     </row>
-    <row r="17"/>
+    <row r="17">
+      <c r="A17" s="55" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B17" s="41" t="n">
+        <v>3222</v>
+      </c>
+    </row>
     <row r="18"/>
     <row r="19"/>
     <row r="20"/>
@@ -3137,7 +3144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3274,7 +3281,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="3">
@@ -3325,7 +3332,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="4">
@@ -3376,7 +3383,7 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="5">
@@ -3427,7 +3434,7 @@
         <v/>
       </c>
       <c r="N5" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="6">
@@ -3478,7 +3485,7 @@
         <v/>
       </c>
       <c r="N6" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="7">
@@ -3529,7 +3536,7 @@
         <v/>
       </c>
       <c r="N7" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="8">
@@ -3558,10 +3565,10 @@
         </is>
       </c>
       <c r="G8" s="52" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H8" s="52" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I8" s="52" t="n">
         <v>2</v>
@@ -3580,7 +3587,7 @@
         <v/>
       </c>
       <c r="N8" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="9">
@@ -3609,10 +3616,10 @@
         </is>
       </c>
       <c r="G9" s="52" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H9" s="52" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I9" s="52" t="n">
         <v>1</v>
@@ -3631,7 +3638,7 @@
         <v/>
       </c>
       <c r="N9" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="10">
@@ -3660,10 +3667,10 @@
         </is>
       </c>
       <c r="G10" s="52" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H10" s="52" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I10" s="52" t="n">
         <v>3</v>
@@ -3682,7 +3689,7 @@
         <v/>
       </c>
       <c r="N10" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="11">
@@ -3711,10 +3718,10 @@
         </is>
       </c>
       <c r="G11" s="52" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H11" s="52" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I11" s="52" t="n">
         <v>1</v>
@@ -3733,7 +3740,7 @@
         <v/>
       </c>
       <c r="N11" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="12">
@@ -3762,10 +3769,10 @@
         </is>
       </c>
       <c r="G12" s="52" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="H12" s="52" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="I12" s="52" t="n">
         <v>0</v>
@@ -3784,7 +3791,7 @@
         <v/>
       </c>
       <c r="N12" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="13">
@@ -3813,10 +3820,10 @@
         </is>
       </c>
       <c r="G13" s="52" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H13" s="52" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="I13" s="52" t="n">
         <v>0</v>
@@ -3835,7 +3842,7 @@
         <v/>
       </c>
       <c r="N13" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="14">
@@ -3864,10 +3871,10 @@
         </is>
       </c>
       <c r="G14" s="52" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="H14" s="52" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="I14" s="52" t="n">
         <v>0</v>
@@ -3886,7 +3893,58 @@
         <v/>
       </c>
       <c r="N14" s="57" t="n">
-        <v>46321</v>
+        <v>46323</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="57" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B15" s="52" t="inlineStr">
+        <is>
+          <t>p16</t>
+        </is>
+      </c>
+      <c r="C15" s="52" t="inlineStr">
+        <is>
+          <t>Флисовый костюм для мальчика</t>
+        </is>
+      </c>
+      <c r="D15" s="52" t="n">
+        <v>485253326</v>
+      </c>
+      <c r="E15" s="52" t="n">
+        <v>2717792690</v>
+      </c>
+      <c r="F15" s="53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/DfDTI9eFHc0/</t>
+        </is>
+      </c>
+      <c r="G15" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="54">
+        <f>IF(N(G15)&gt;0,(I15+J15+K15+L15)/G15,"")</f>
+        <v/>
+      </c>
+      <c r="N15" s="57" t="n">
+        <v>46323</v>
       </c>
     </row>
   </sheetData>
@@ -3904,6 +3962,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId14"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Посты Instagram и Telegram: 2026-10-30
</commit_message>
<xml_diff>
--- a/bot/ivbaby-promo.xlsx
+++ b/bot/ivbaby-promo.xlsx
@@ -498,12 +498,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Динамика'!$A$2:$A$17</f>
+              <f>'Динамика'!$A$2:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Динамика'!$B$2:$B$17</f>
+              <f>'Динамика'!$B$2:$B$18</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -676,12 +676,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Наши посты'!$B$2:$B$15</f>
+              <f>'Наши посты'!$B$2:$B$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Наши посты'!$G$2:$G$15</f>
+              <f>'Наши посты'!$G$2:$G$16</f>
             </numRef>
           </val>
         </ser>
@@ -1701,7 +1701,14 @@
         <v>3222</v>
       </c>
     </row>
-    <row r="18"/>
+    <row r="18">
+      <c r="A18" s="55" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B18" s="41" t="n">
+        <v>3222</v>
+      </c>
+    </row>
     <row r="19"/>
     <row r="20"/>
     <row r="21"/>
@@ -3144,7 +3151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -3259,10 +3266,10 @@
         </is>
       </c>
       <c r="G2" s="48" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H2" s="48" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="I2" s="48" t="n">
         <v>3</v>
@@ -3281,7 +3288,7 @@
         <v/>
       </c>
       <c r="N2" s="56" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="3">
@@ -3310,10 +3317,10 @@
         </is>
       </c>
       <c r="G3" s="52" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H3" s="52" t="n">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I3" s="52" t="n">
         <v>3</v>
@@ -3332,7 +3339,7 @@
         <v/>
       </c>
       <c r="N3" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="4">
@@ -3361,7 +3368,7 @@
         </is>
       </c>
       <c r="G4" s="52" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H4" s="52" t="n">
         <v>63</v>
@@ -3383,7 +3390,7 @@
         <v/>
       </c>
       <c r="N4" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="5">
@@ -3412,10 +3419,10 @@
         </is>
       </c>
       <c r="G5" s="52" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H5" s="52" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I5" s="52" t="n">
         <v>2</v>
@@ -3434,7 +3441,7 @@
         <v/>
       </c>
       <c r="N5" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="6">
@@ -3463,10 +3470,10 @@
         </is>
       </c>
       <c r="G6" s="52" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H6" s="52" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I6" s="52" t="n">
         <v>0</v>
@@ -3485,7 +3492,7 @@
         <v/>
       </c>
       <c r="N6" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="7">
@@ -3514,7 +3521,7 @@
         </is>
       </c>
       <c r="G7" s="52" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H7" s="52" t="n">
         <v>43</v>
@@ -3536,7 +3543,7 @@
         <v/>
       </c>
       <c r="N7" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="8">
@@ -3565,10 +3572,10 @@
         </is>
       </c>
       <c r="G8" s="52" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H8" s="52" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I8" s="52" t="n">
         <v>2</v>
@@ -3587,7 +3594,7 @@
         <v/>
       </c>
       <c r="N8" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="9">
@@ -3616,10 +3623,10 @@
         </is>
       </c>
       <c r="G9" s="52" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H9" s="52" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I9" s="52" t="n">
         <v>1</v>
@@ -3638,7 +3645,7 @@
         <v/>
       </c>
       <c r="N9" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="10">
@@ -3670,7 +3677,7 @@
         <v>31</v>
       </c>
       <c r="H10" s="52" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I10" s="52" t="n">
         <v>3</v>
@@ -3689,7 +3696,7 @@
         <v/>
       </c>
       <c r="N10" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="11">
@@ -3718,10 +3725,10 @@
         </is>
       </c>
       <c r="G11" s="52" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H11" s="52" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="I11" s="52" t="n">
         <v>1</v>
@@ -3740,7 +3747,7 @@
         <v/>
       </c>
       <c r="N11" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="12">
@@ -3769,10 +3776,10 @@
         </is>
       </c>
       <c r="G12" s="52" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H12" s="52" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="I12" s="52" t="n">
         <v>0</v>
@@ -3791,7 +3798,7 @@
         <v/>
       </c>
       <c r="N12" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="13">
@@ -3820,10 +3827,10 @@
         </is>
       </c>
       <c r="G13" s="52" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H13" s="52" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="I13" s="52" t="n">
         <v>0</v>
@@ -3842,7 +3849,7 @@
         <v/>
       </c>
       <c r="N13" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="14">
@@ -3871,13 +3878,13 @@
         </is>
       </c>
       <c r="G14" s="52" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H14" s="52" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="I14" s="52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" s="52" t="n">
         <v>0</v>
@@ -3893,7 +3900,7 @@
         <v/>
       </c>
       <c r="N14" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="15">
@@ -3922,13 +3929,13 @@
         </is>
       </c>
       <c r="G15" s="52" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="H15" s="52" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="I15" s="52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" s="52" t="n">
         <v>0</v>
@@ -3937,14 +3944,65 @@
         <v>0</v>
       </c>
       <c r="L15" s="52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15" s="54">
         <f>IF(N(G15)&gt;0,(I15+J15+K15+L15)/G15,"")</f>
         <v/>
       </c>
       <c r="N15" s="57" t="n">
-        <v>46323</v>
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="57" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B16" s="52" t="inlineStr">
+        <is>
+          <t>p17</t>
+        </is>
+      </c>
+      <c r="C16" s="52" t="inlineStr">
+        <is>
+          <t>Шпаргалка: уход за вещами с начёсом</t>
+        </is>
+      </c>
+      <c r="D16" s="52" t="n">
+        <v>147321676</v>
+      </c>
+      <c r="E16" s="52" t="n">
+        <v>1097457144</v>
+      </c>
+      <c r="F16" s="53" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DfIZoHQAVxH/</t>
+        </is>
+      </c>
+      <c r="G16" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="54">
+        <f>IF(N(G16)&gt;0,(I16+J16+K16+L16)/G16,"")</f>
+        <v/>
+      </c>
+      <c r="N16" s="57" t="n">
+        <v>46325</v>
       </c>
     </row>
   </sheetData>
@@ -3963,6 +4021,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId15"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>